<commit_message>
Site_Definition_Cleanup: apply Arthur's site file fixes from issue #38
Add missing required columns (Compressors, Gas Lift, Dehydrators, VRUs)
with suggested default values. Remove excluded unrecognized columns from
Dehydrators tab in AllEquipment.xlsx. Validation findings: 74 → 43.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input/Studies/C3/C3_Prototypical_Sites/C3_Example_Site.xlsx
+++ b/input/Studies/C3/C3_Prototypical_Sites/C3_Example_Site.xlsx
@@ -1057,24 +1057,24 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="62" t="inlineStr">
         <is>
           <t>maesVersion</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="62" t="inlineStr">
         <is>
           <t>0.4.0</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="62" t="inlineStr">
         <is>
           <t>gitDescribe</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="62" t="inlineStr">
         <is>
           <t>v0.2.0-185-g1ee2031-dirty</t>
         </is>
@@ -1381,12 +1381,12 @@
           <t>Model ID</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="62" t="inlineStr">
         <is>
           <t>Operator</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="62" t="inlineStr">
         <is>
           <t>Prototypical Site Number</t>
         </is>
@@ -1414,12 +1414,12 @@
           <t>Facility.json</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="62" t="inlineStr">
         <is>
           <t>MAES</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="62" t="inlineStr">
         <is>
           <t>MAES</t>
         </is>
@@ -3687,7 +3687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AZ5"/>
+  <dimension ref="A1:BC5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="62" min="1" max="1"/>
@@ -3979,6 +3979,21 @@
           <t>Factor Tag</t>
         </is>
       </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>CCEE Ratio Distribution</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>Compressor Efficiency</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>Crankcase Emissions Flag</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1" s="63">
       <c r="A2" s="62" t="inlineStr">
@@ -4161,6 +4176,15 @@
           <t>wellpad_compressor_0to200HP</t>
         </is>
       </c>
+      <c r="BA2" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="BC2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1" s="63">
       <c r="A3" s="62" t="inlineStr">
@@ -4343,6 +4367,15 @@
           <t>wellpad_compressor_0to200HP</t>
         </is>
       </c>
+      <c r="BA3" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="BB3" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="BC3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1" s="63">
       <c r="A4" s="62" t="inlineStr">
@@ -4525,6 +4558,15 @@
           <t>wellpad_compressor_0to200HP</t>
         </is>
       </c>
+      <c r="BA4" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="BC4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" ht="14.25" customHeight="1" s="63">
       <c r="A5" s="62" t="inlineStr">
@@ -4706,6 +4748,15 @@
         <is>
           <t>wellpad_compressor_0to200HP</t>
         </is>
+      </c>
+      <c r="BA5" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="BB5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="BC5" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>